<commit_message>
agentic-qe-mvp: learning off by default (AQE_LEARNING=on); Learning and Test Lab out of the menu; Reporting and Traceability under MVP demo; read-only Home
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-eqe-CYC-1/08-report/CYC-1-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-eqe-CYC-1/08-report/CYC-1-cycle-report.xlsx
@@ -19,14 +19,13 @@
     <sheet sheetId="13" name="Approvals" state="visible" r:id="rId16"/>
     <sheet sheetId="14" name="Skills" state="visible" r:id="rId17"/>
     <sheet sheetId="15" name="Hand-overs" state="visible" r:id="rId18"/>
-    <sheet sheetId="16" name="Adapted this cycle" state="visible" r:id="rId19"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2528" uniqueCount="930">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2526" uniqueCount="929">
   <si>
     <t>Metric</t>
   </si>
@@ -178,7 +177,7 @@
     <t>github</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) at 2026-10-11T16:15:17.679Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) at 2026-10-11T16:44:09.579Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -2571,7 +2570,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-11T16:15:18.665Z</t>
+    <t>2026-10-11T16:44:10.301Z</t>
   </si>
   <si>
     <t>118 requirements approved; 10 excluded (gaps AQPI-8, AQPI-13, AQPI-22); 0 conflict(s) resolved</t>
@@ -2833,9 +2832,6 @@
   </si>
   <si>
     <t>cycleReport: delivered; comparison: n/a; testCaseExport: delivered</t>
-  </si>
-  <si>
-    <t>Lesson applied</t>
   </si>
 </sst>
 </file>
@@ -5740,29 +5736,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="2" width="110" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>929</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>837</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E4"/>
@@ -11262,7 +11235,7 @@
         <v>669</v>
       </c>
       <c r="E2" s="2">
-        <v>1231</v>
+        <v>1038</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -11281,7 +11254,7 @@
         <v>669</v>
       </c>
       <c r="E3" s="2">
-        <v>160</v>
+        <v>108</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -11300,7 +11273,7 @@
         <v>669</v>
       </c>
       <c r="E4" s="2">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -11319,7 +11292,7 @@
         <v>669</v>
       </c>
       <c r="E5" s="2">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -11338,7 +11311,7 @@
         <v>669</v>
       </c>
       <c r="E6" s="2">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -11357,7 +11330,7 @@
         <v>669</v>
       </c>
       <c r="E7" s="2">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -11376,7 +11349,7 @@
         <v>669</v>
       </c>
       <c r="E8" s="2">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -11416,7 +11389,7 @@
         <v>669</v>
       </c>
       <c r="E10" s="2">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>

</xml_diff>

<commit_message>
agentic-qe-mvp: reviewer decides only code gaps and conflicts; gap defects carry story, epic, criteria, reviewer and a Jira payload
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-eqe-CYC-1/08-report/CYC-1-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-eqe-CYC-1/08-report/CYC-1-cycle-report.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2526" uniqueCount="929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2526" uniqueCount="931">
   <si>
     <t>Metric</t>
   </si>
@@ -177,7 +177,7 @@
     <t>github</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) at 2026-10-11T16:44:09.579Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) at 2026-10-11T17:06:39.764Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -2111,13 +2111,13 @@
     <t>AQPI-8</t>
   </si>
   <si>
-    <t>not raised in Jira</t>
-  </si>
-  <si>
-    <t>Code implements AQPI-8 (4 acceptance criteria)</t>
-  </si>
-  <si>
-    <t>No code in demo/hotel-booking-platform mentions AQPI-8</t>
+    <t>not raised in Jira; linked to AQPI-8 in the platform</t>
+  </si>
+  <si>
+    <t>The code implements AQPI-8 4.2 Sort and filter hotel results (4 acceptance criteria)</t>
+  </si>
+  <si>
+    <t>No code in sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) mentions AQPI-8</t>
   </si>
   <si>
     <t>DEF-002</t>
@@ -2129,10 +2129,13 @@
     <t>AQPI-13</t>
   </si>
   <si>
-    <t>Code implements AQPI-13 (3 acceptance criteria)</t>
-  </si>
-  <si>
-    <t>No code in demo/hotel-booking-platform mentions AQPI-13</t>
+    <t>not raised in Jira; linked to AQPI-13 in the platform</t>
+  </si>
+  <si>
+    <t>The code implements AQPI-13 5.3 Explain and control personalization (3 acceptance criteria)</t>
+  </si>
+  <si>
+    <t>No code in sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) mentions AQPI-13</t>
   </si>
   <si>
     <t>DEF-003</t>
@@ -2144,10 +2147,13 @@
     <t>AQPI-22</t>
   </si>
   <si>
-    <t>Code implements AQPI-22 (3 acceptance criteria)</t>
-  </si>
-  <si>
-    <t>No code in demo/hotel-booking-platform mentions AQPI-22</t>
+    <t>not raised in Jira; linked to AQPI-22 in the platform</t>
+  </si>
+  <si>
+    <t>The code implements AQPI-22 7.4 Show booking outcome (3 acceptance criteria)</t>
+  </si>
+  <si>
+    <t>No code in sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) mentions AQPI-22</t>
   </si>
   <si>
     <t>First seen</t>
@@ -2570,7 +2576,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-11T16:44:10.301Z</t>
+    <t>2026-10-11T17:06:40.510Z</t>
   </si>
   <si>
     <t>118 requirements approved; 10 excluded (gaps AQPI-8, AQPI-13, AQPI-22); 0 conflict(s) resolved</t>
@@ -3426,19 +3432,19 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>12</v>
@@ -3467,16 +3473,16 @@
         <v>41</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="F2" s="2">
         <v>6</v>
@@ -3497,24 +3503,24 @@
         <v>71</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
     </row>
     <row r="3" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="F3" s="2">
         <v>0</v>
@@ -3535,7 +3541,7 @@
         <v>71</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3543,16 +3549,16 @@
         <v>120</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="F4" s="2">
         <v>0</v>
@@ -3573,7 +3579,7 @@
         <v>71</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="5" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3581,16 +3587,16 @@
         <v>150</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="F5" s="2">
         <v>1</v>
@@ -3611,7 +3617,7 @@
         <v>71</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
     <row r="6" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3619,16 +3625,16 @@
         <v>171</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
       <c r="F6" s="2">
         <v>0</v>
@@ -3649,24 +3655,24 @@
         <v>71</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="7" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>766</v>
+        <v>768</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -3687,7 +3693,7 @@
         <v>71</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="8" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3695,16 +3701,16 @@
         <v>183</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="F8" s="2">
         <v>0</v>
@@ -3725,7 +3731,7 @@
         <v>71</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="9" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3733,16 +3739,16 @@
         <v>687</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>768</v>
+        <v>770</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
@@ -3763,7 +3769,7 @@
         <v>71</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="10" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3771,16 +3777,16 @@
         <v>204</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>769</v>
+        <v>771</v>
       </c>
       <c r="F10" s="2">
         <v>0</v>
@@ -3801,24 +3807,24 @@
         <v>71</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="11" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
@@ -3839,7 +3845,7 @@
         <v>71</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="12" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3847,16 +3853,16 @@
         <v>221</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>772</v>
+        <v>774</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
@@ -3877,7 +3883,7 @@
         <v>71</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="13" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3885,16 +3891,16 @@
         <v>250</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>773</v>
+        <v>775</v>
       </c>
       <c r="F13" s="2">
         <v>1</v>
@@ -3915,7 +3921,7 @@
         <v>71</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
     </row>
     <row r="14" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3923,16 +3929,16 @@
         <v>693</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>770</v>
+        <v>772</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>774</v>
+        <v>776</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
@@ -3953,24 +3959,24 @@
         <v>71</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="15" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>776</v>
+        <v>778</v>
       </c>
       <c r="F15" s="2">
         <v>0</v>
@@ -3991,7 +3997,7 @@
         <v>71</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="16" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -3999,16 +4005,16 @@
         <v>265</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>777</v>
+        <v>779</v>
       </c>
       <c r="F16" s="2">
         <v>0</v>
@@ -4029,7 +4035,7 @@
         <v>71</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="17" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4037,16 +4043,16 @@
         <v>286</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>778</v>
+        <v>780</v>
       </c>
       <c r="F17" s="2">
         <v>0</v>
@@ -4067,7 +4073,7 @@
         <v>71</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="18" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4075,16 +4081,16 @@
         <v>303</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>775</v>
+        <v>777</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>779</v>
+        <v>781</v>
       </c>
       <c r="F18" s="2">
         <v>0</v>
@@ -4105,24 +4111,24 @@
         <v>71</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="19" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>781</v>
+        <v>783</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -4143,7 +4149,7 @@
         <v>71</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="20" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4151,16 +4157,16 @@
         <v>324</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>782</v>
+        <v>784</v>
       </c>
       <c r="F20" s="2">
         <v>0</v>
@@ -4181,7 +4187,7 @@
         <v>71</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="21" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4189,16 +4195,16 @@
         <v>349</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>783</v>
+        <v>785</v>
       </c>
       <c r="F21" s="2">
         <v>0</v>
@@ -4219,7 +4225,7 @@
         <v>71</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="22" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4227,16 +4233,16 @@
         <v>374</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>784</v>
+        <v>786</v>
       </c>
       <c r="F22" s="2">
         <v>0</v>
@@ -4257,24 +4263,24 @@
         <v>71</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="23" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>780</v>
+        <v>782</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>785</v>
+        <v>787</v>
       </c>
       <c r="F23" s="2">
         <v>0</v>
@@ -4295,24 +4301,24 @@
         <v>71</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="24" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>787</v>
+        <v>789</v>
       </c>
       <c r="F24" s="2">
         <v>0</v>
@@ -4333,7 +4339,7 @@
         <v>71</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="25" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4341,16 +4347,16 @@
         <v>399</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>788</v>
+        <v>790</v>
       </c>
       <c r="F25" s="2">
         <v>1</v>
@@ -4371,7 +4377,7 @@
         <v>71</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
     <row r="26" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4379,16 +4385,16 @@
         <v>418</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>789</v>
+        <v>791</v>
       </c>
       <c r="F26" s="2">
         <v>0</v>
@@ -4409,7 +4415,7 @@
         <v>71</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="27" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4417,16 +4423,16 @@
         <v>439</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>786</v>
+        <v>788</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>790</v>
+        <v>792</v>
       </c>
       <c r="F27" s="2">
         <v>0</v>
@@ -4447,24 +4453,24 @@
         <v>71</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="28" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>41</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>792</v>
+        <v>794</v>
       </c>
       <c r="F28" s="2">
         <v>0</v>
@@ -4485,7 +4491,7 @@
         <v>71</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="29" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4493,16 +4499,16 @@
         <v>452</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>793</v>
+        <v>795</v>
       </c>
       <c r="F29" s="2">
         <v>0</v>
@@ -4523,7 +4529,7 @@
         <v>71</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="30" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4531,16 +4537,16 @@
         <v>472</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>794</v>
+        <v>796</v>
       </c>
       <c r="F30" s="2">
         <v>1</v>
@@ -4561,7 +4567,7 @@
         <v>71</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
     <row r="31" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4569,16 +4575,16 @@
         <v>497</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>795</v>
+        <v>797</v>
       </c>
       <c r="F31" s="2">
         <v>1</v>
@@ -4599,7 +4605,7 @@
         <v>71</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
     <row r="32" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -4607,16 +4613,16 @@
         <v>514</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>791</v>
+        <v>793</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>796</v>
+        <v>798</v>
       </c>
       <c r="F32" s="2">
         <v>1</v>
@@ -4637,7 +4643,7 @@
         <v>71</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
   </sheetData>
@@ -4672,13 +4678,13 @@
         <v>53</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>797</v>
+        <v>799</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>57</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>798</v>
+        <v>800</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>567</v>
@@ -4687,19 +4693,19 @@
         <v>54</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>800</v>
+        <v>802</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>801</v>
+        <v>803</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>665</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>802</v>
+        <v>804</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>675</v>
@@ -4731,10 +4737,10 @@
         <v>590</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>803</v>
+        <v>805</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="K2" s="2" t="s">
         <v>669</v>
@@ -4772,10 +4778,10 @@
         <v>590</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>805</v>
+        <v>807</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>804</v>
+        <v>806</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>669</v>
@@ -4813,10 +4819,10 @@
         <v>590</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>806</v>
+        <v>808</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>807</v>
+        <v>809</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>669</v>
@@ -4854,10 +4860,10 @@
         <v>590</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>808</v>
+        <v>810</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>809</v>
+        <v>811</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>669</v>
@@ -4895,10 +4901,10 @@
         <v>590</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>811</v>
+        <v>813</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>669</v>
@@ -4936,10 +4942,10 @@
         <v>590</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>812</v>
+        <v>814</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>813</v>
+        <v>815</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>669</v>
@@ -4977,10 +4983,10 @@
         <v>590</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>814</v>
+        <v>816</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>815</v>
+        <v>817</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>669</v>
@@ -5018,7 +5024,7 @@
         <v>645</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>816</v>
+        <v>818</v>
       </c>
       <c r="J9" s="2"/>
       <c r="K9" s="2" t="s">
@@ -5057,10 +5063,10 @@
         <v>590</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>817</v>
+        <v>819</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>818</v>
+        <v>820</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>669</v>
@@ -5098,7 +5104,7 @@
         <v>645</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>819</v>
+        <v>821</v>
       </c>
       <c r="J11" s="2"/>
       <c r="K11" s="2" t="s">
@@ -5137,7 +5143,7 @@
         <v>645</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>820</v>
+        <v>822</v>
       </c>
       <c r="J12" s="2"/>
       <c r="K12" s="2" t="s">
@@ -5176,7 +5182,7 @@
         <v>645</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>821</v>
+        <v>823</v>
       </c>
       <c r="J13" s="2"/>
       <c r="K13" s="2" t="s">
@@ -5215,7 +5221,7 @@
         <v>645</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>822</v>
+        <v>824</v>
       </c>
       <c r="J14" s="2"/>
       <c r="K14" s="2" t="s">
@@ -5252,40 +5258,40 @@
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>823</v>
+        <v>825</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>824</v>
+        <v>826</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>825</v>
+        <v>827</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>826</v>
+        <v>828</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>828</v>
+        <v>830</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>829</v>
+        <v>831</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>830</v>
+        <v>832</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>831</v>
+        <v>833</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>832</v>
+        <v>834</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>667</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>833</v>
+        <v>835</v>
       </c>
     </row>
   </sheetData>
@@ -5308,36 +5314,36 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>835</v>
+        <v>837</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>836</v>
+        <v>838</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>827</v>
+        <v>829</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>837</v>
+        <v>839</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>838</v>
+        <v>840</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>839</v>
+        <v>841</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>840</v>
+        <v>842</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>841</v>
+        <v>843</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>842</v>
+        <v>844</v>
       </c>
     </row>
   </sheetData>
@@ -5360,189 +5366,189 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>843</v>
+        <v>845</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>567</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>844</v>
+        <v>846</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>845</v>
+        <v>847</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>846</v>
+        <v>848</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>847</v>
+        <v>849</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>848</v>
+        <v>850</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>849</v>
+        <v>851</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>850</v>
+        <v>852</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>851</v>
+        <v>853</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>852</v>
+        <v>854</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>853</v>
+        <v>855</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>854</v>
+        <v>856</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>855</v>
+        <v>857</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>856</v>
+        <v>858</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>857</v>
+        <v>859</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>858</v>
+        <v>860</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>859</v>
+        <v>861</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>860</v>
+        <v>862</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>861</v>
+        <v>863</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>862</v>
+        <v>864</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>863</v>
+        <v>865</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>864</v>
+        <v>866</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>865</v>
+        <v>867</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>866</v>
+        <v>868</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>867</v>
+        <v>869</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>868</v>
+        <v>870</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>869</v>
+        <v>871</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>870</v>
+        <v>872</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>872</v>
+        <v>874</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>873</v>
+        <v>875</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>874</v>
+        <v>876</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>875</v>
+        <v>877</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>876</v>
+        <v>878</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>877</v>
+        <v>879</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>878</v>
+        <v>880</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>879</v>
+        <v>881</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>880</v>
+        <v>882</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>881</v>
+        <v>883</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>882</v>
+        <v>884</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>883</v>
+        <v>885</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>884</v>
+        <v>886</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>885</v>
+        <v>887</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>886</v>
+        <v>888</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>887</v>
+        <v>889</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>888</v>
+        <v>890</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>889</v>
+        <v>891</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>890</v>
+        <v>892</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>891</v>
+        <v>893</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>892</v>
+        <v>894</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>893</v>
+        <v>895</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>894</v>
+        <v>896</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>895</v>
+        <v>897</v>
       </c>
     </row>
   </sheetData>
@@ -5565,169 +5571,169 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>896</v>
+        <v>898</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>897</v>
+        <v>899</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>898</v>
+        <v>900</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>899</v>
+        <v>901</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>900</v>
+        <v>902</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>902</v>
+        <v>904</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>904</v>
+        <v>906</v>
       </c>
     </row>
     <row r="3" spans="2:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>871</v>
+        <v>873</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>905</v>
+        <v>907</v>
       </c>
     </row>
     <row r="4" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>906</v>
+        <v>908</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>907</v>
+        <v>909</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>908</v>
+        <v>910</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>909</v>
+        <v>911</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>910</v>
+        <v>912</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>911</v>
+        <v>913</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>912</v>
+        <v>914</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>913</v>
+        <v>915</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>914</v>
+        <v>916</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>915</v>
+        <v>917</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>916</v>
+        <v>918</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>917</v>
+        <v>919</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>918</v>
+        <v>920</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>919</v>
+        <v>921</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>920</v>
+        <v>922</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>921</v>
+        <v>923</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>922</v>
+        <v>924</v>
       </c>
     </row>
     <row r="9" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>923</v>
+        <v>925</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>924</v>
+        <v>926</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>925</v>
+        <v>927</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>926</v>
+        <v>928</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>927</v>
+        <v>929</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>903</v>
+        <v>905</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>71</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>928</v>
+        <v>930</v>
       </c>
     </row>
   </sheetData>
@@ -11235,7 +11241,7 @@
         <v>669</v>
       </c>
       <c r="E2" s="2">
-        <v>1038</v>
+        <v>1091</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -11254,7 +11260,7 @@
         <v>669</v>
       </c>
       <c r="E3" s="2">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -11273,7 +11279,7 @@
         <v>669</v>
       </c>
       <c r="E4" s="2">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -11292,7 +11298,7 @@
         <v>669</v>
       </c>
       <c r="E5" s="2">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -11311,7 +11317,7 @@
         <v>669</v>
       </c>
       <c r="E6" s="2">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -11330,7 +11336,7 @@
         <v>669</v>
       </c>
       <c r="E7" s="2">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -11349,7 +11355,7 @@
         <v>669</v>
       </c>
       <c r="E8" s="2">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -11389,7 +11395,7 @@
         <v>669</v>
       </c>
       <c r="E10" s="2">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -11595,15 +11601,15 @@
         <v>693</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>73</v>
@@ -11615,27 +11621,27 @@
     </row>
     <row r="4" spans="1:15" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>686</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>688</v>
+        <v>700</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>73</v>
@@ -11677,10 +11683,10 @@
         <v>664</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>665</v>
@@ -11689,7 +11695,7 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
     </row>
   </sheetData>
@@ -11716,16 +11722,16 @@
         <v>53</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>590</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>23</v>
@@ -11754,7 +11760,7 @@
         <v>0</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11777,7 +11783,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11800,7 +11806,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11823,7 +11829,7 @@
         <v>0</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11846,7 +11852,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11869,7 +11875,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11892,7 +11898,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11915,7 +11921,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11938,7 +11944,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11961,7 +11967,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -11984,7 +11990,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12007,7 +12013,7 @@
         <v>0</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12030,7 +12036,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12053,7 +12059,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12076,7 +12082,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12099,7 +12105,7 @@
         <v>0</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12122,7 +12128,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12145,7 +12151,7 @@
         <v>0</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12168,7 +12174,7 @@
         <v>0</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="21" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12191,7 +12197,7 @@
         <v>0</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12214,7 +12220,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="23" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12237,7 +12243,7 @@
         <v>0</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="24" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12260,7 +12266,7 @@
         <v>0</v>
       </c>
       <c r="G24" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12283,7 +12289,7 @@
         <v>0</v>
       </c>
       <c r="G25" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12306,7 +12312,7 @@
         <v>0</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12329,7 +12335,7 @@
         <v>0</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="28" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12352,7 +12358,7 @@
         <v>0</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="29" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12375,7 +12381,7 @@
         <v>0</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="30" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12398,7 +12404,7 @@
         <v>0</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12421,7 +12427,7 @@
         <v>0</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12444,7 +12450,7 @@
         <v>0</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12467,7 +12473,7 @@
         <v>0</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12490,7 +12496,7 @@
         <v>0</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12513,7 +12519,7 @@
         <v>0</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12536,7 +12542,7 @@
         <v>0</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12559,7 +12565,7 @@
         <v>0</v>
       </c>
       <c r="G37" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="38" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12582,7 +12588,7 @@
         <v>0</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="39" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12605,7 +12611,7 @@
         <v>0</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="40" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12628,7 +12634,7 @@
         <v>0</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="41" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12651,7 +12657,7 @@
         <v>0</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="42" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12674,7 +12680,7 @@
         <v>0</v>
       </c>
       <c r="G42" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="43" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12697,7 +12703,7 @@
         <v>0</v>
       </c>
       <c r="G43" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="44" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12720,7 +12726,7 @@
         <v>0</v>
       </c>
       <c r="G44" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="45" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12743,7 +12749,7 @@
         <v>0</v>
       </c>
       <c r="G45" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="46" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12766,7 +12772,7 @@
         <v>0</v>
       </c>
       <c r="G46" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="47" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12789,7 +12795,7 @@
         <v>0</v>
       </c>
       <c r="G47" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="48" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12812,7 +12818,7 @@
         <v>0</v>
       </c>
       <c r="G48" s="2" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
     </row>
     <row r="49" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12835,7 +12841,7 @@
         <v>0</v>
       </c>
       <c r="G49" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="50" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12858,7 +12864,7 @@
         <v>0</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="51" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12881,7 +12887,7 @@
         <v>0</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="52" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12904,7 +12910,7 @@
         <v>0</v>
       </c>
       <c r="G52" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="53" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12927,7 +12933,7 @@
         <v>0</v>
       </c>
       <c r="G53" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="54" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12950,7 +12956,7 @@
         <v>0</v>
       </c>
       <c r="G54" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="55" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12973,7 +12979,7 @@
         <v>0</v>
       </c>
       <c r="G55" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="56" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -12996,7 +13002,7 @@
         <v>0</v>
       </c>
       <c r="G56" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="57" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13019,7 +13025,7 @@
         <v>0</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="58" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13042,7 +13048,7 @@
         <v>0</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="59" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13065,7 +13071,7 @@
         <v>0</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="60" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13088,7 +13094,7 @@
         <v>0</v>
       </c>
       <c r="G60" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="61" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13111,7 +13117,7 @@
         <v>0</v>
       </c>
       <c r="G61" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="62" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13134,7 +13140,7 @@
         <v>0</v>
       </c>
       <c r="G62" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="63" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13157,7 +13163,7 @@
         <v>0</v>
       </c>
       <c r="G63" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="64" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13180,7 +13186,7 @@
         <v>0</v>
       </c>
       <c r="G64" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="65" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13203,7 +13209,7 @@
         <v>0</v>
       </c>
       <c r="G65" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="66" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13226,7 +13232,7 @@
         <v>0</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="67" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13249,7 +13255,7 @@
         <v>0</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="68" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13272,7 +13278,7 @@
         <v>0</v>
       </c>
       <c r="G68" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="69" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13295,7 +13301,7 @@
         <v>0</v>
       </c>
       <c r="G69" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="70" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13318,7 +13324,7 @@
         <v>0</v>
       </c>
       <c r="G70" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="71" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13341,7 +13347,7 @@
         <v>0</v>
       </c>
       <c r="G71" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="72" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13364,7 +13370,7 @@
         <v>0</v>
       </c>
       <c r="G72" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="73" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13387,7 +13393,7 @@
         <v>0</v>
       </c>
       <c r="G73" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="74" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13410,7 +13416,7 @@
         <v>0</v>
       </c>
       <c r="G74" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="75" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13433,7 +13439,7 @@
         <v>0</v>
       </c>
       <c r="G75" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="76" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13456,7 +13462,7 @@
         <v>0</v>
       </c>
       <c r="G76" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="77" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13479,7 +13485,7 @@
         <v>0</v>
       </c>
       <c r="G77" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="78" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13502,7 +13508,7 @@
         <v>0</v>
       </c>
       <c r="G78" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="79" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13525,7 +13531,7 @@
         <v>0</v>
       </c>
       <c r="G79" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="80" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13548,7 +13554,7 @@
         <v>0</v>
       </c>
       <c r="G80" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="81" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13571,7 +13577,7 @@
         <v>0</v>
       </c>
       <c r="G81" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="82" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13594,7 +13600,7 @@
         <v>0</v>
       </c>
       <c r="G82" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="83" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13617,7 +13623,7 @@
         <v>0</v>
       </c>
       <c r="G83" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="84" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13640,7 +13646,7 @@
         <v>0</v>
       </c>
       <c r="G84" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="85" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13663,7 +13669,7 @@
         <v>0</v>
       </c>
       <c r="G85" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="86" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13686,7 +13692,7 @@
         <v>0</v>
       </c>
       <c r="G86" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="87" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13709,7 +13715,7 @@
         <v>0</v>
       </c>
       <c r="G87" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="88" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13732,7 +13738,7 @@
         <v>0</v>
       </c>
       <c r="G88" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="89" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13755,7 +13761,7 @@
         <v>0</v>
       </c>
       <c r="G89" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="90" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13778,7 +13784,7 @@
         <v>0</v>
       </c>
       <c r="G90" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="91" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13801,7 +13807,7 @@
         <v>0</v>
       </c>
       <c r="G91" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="92" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13824,7 +13830,7 @@
         <v>0</v>
       </c>
       <c r="G92" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="93" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13847,7 +13853,7 @@
         <v>0</v>
       </c>
       <c r="G93" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="94" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13870,7 +13876,7 @@
         <v>0</v>
       </c>
       <c r="G94" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="95" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13893,7 +13899,7 @@
         <v>0</v>
       </c>
       <c r="G95" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="96" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13916,7 +13922,7 @@
         <v>0</v>
       </c>
       <c r="G96" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="97" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13939,7 +13945,7 @@
         <v>0</v>
       </c>
       <c r="G97" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="98" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13962,7 +13968,7 @@
         <v>0</v>
       </c>
       <c r="G98" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="99" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -13985,7 +13991,7 @@
         <v>0</v>
       </c>
       <c r="G99" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="100" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14008,7 +14014,7 @@
         <v>0</v>
       </c>
       <c r="G100" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="101" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14031,7 +14037,7 @@
         <v>0</v>
       </c>
       <c r="G101" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="102" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14054,7 +14060,7 @@
         <v>0</v>
       </c>
       <c r="G102" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="103" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14077,7 +14083,7 @@
         <v>0</v>
       </c>
       <c r="G103" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="104" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14100,7 +14106,7 @@
         <v>0</v>
       </c>
       <c r="G104" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="105" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14123,7 +14129,7 @@
         <v>0</v>
       </c>
       <c r="G105" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="106" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14146,7 +14152,7 @@
         <v>0</v>
       </c>
       <c r="G106" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="107" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14169,7 +14175,7 @@
         <v>0</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="108" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14192,7 +14198,7 @@
         <v>0</v>
       </c>
       <c r="G108" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="109" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14215,7 +14221,7 @@
         <v>0</v>
       </c>
       <c r="G109" s="2" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
     </row>
     <row r="110" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14238,7 +14244,7 @@
         <v>0</v>
       </c>
       <c r="G110" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="111" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14261,7 +14267,7 @@
         <v>0</v>
       </c>
       <c r="G111" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="112" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14284,7 +14290,7 @@
         <v>0</v>
       </c>
       <c r="G112" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="113" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14307,7 +14313,7 @@
         <v>0</v>
       </c>
       <c r="G113" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="114" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14330,7 +14336,7 @@
         <v>0</v>
       </c>
       <c r="G114" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="115" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14353,7 +14359,7 @@
         <v>0</v>
       </c>
       <c r="G115" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="116" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14376,7 +14382,7 @@
         <v>0</v>
       </c>
       <c r="G116" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="117" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14399,7 +14405,7 @@
         <v>0</v>
       </c>
       <c r="G117" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="118" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14422,7 +14428,7 @@
         <v>0</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
     <row r="119" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -14445,7 +14451,7 @@
         <v>0</v>
       </c>
       <c r="G119" s="2" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
     </row>
   </sheetData>
@@ -14467,13 +14473,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>6</v>
@@ -14481,212 +14487,212 @@
     </row>
     <row r="2" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>723</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>721</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>719</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>592</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="13" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="14" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="15" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>71</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
     </row>
     <row r="16" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>614</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
agentic-qe-mvp: capability catalogue on Home, Functional shown as DQE, track sign-off owner, exit criteria and evidence check, EQE journey traceability
Co-Authored-By: Devin AI <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/agentic-qe-mvp/demo-artifacts/flow-1-hotel-eqe-CYC-1/08-report/CYC-1-cycle-report.xlsx
+++ b/agentic-qe-mvp/demo-artifacts/flow-1-hotel-eqe-CYC-1/08-report/CYC-1-cycle-report.xlsx
@@ -87,7 +87,7 @@
     <t>{"functional":8,"eqe":13,"automation":8,"non-functional":5}</t>
   </si>
   <si>
-    <t>Scripts</t>
+    <t>Automation scripts</t>
   </si>
   <si>
     <t>Executed (real)</t>
@@ -177,7 +177,7 @@
     <t>github</t>
   </si>
   <si>
-    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) at 2026-10-11T17:06:39.764Z</t>
+    <t>Pulled live from GitHub: git clone of sri465inno/uc-agentic-quality-engineering@demo/hotel-booking-platform (b212a32) at 2026-10-12T01:34:58.194Z</t>
   </si>
   <si>
     <t>ID</t>
@@ -2576,7 +2576,7 @@
     <t>Priya Shah</t>
   </si>
   <si>
-    <t>2026-10-11T17:06:40.510Z</t>
+    <t>2026-10-12T01:34:58.838Z</t>
   </si>
   <si>
     <t>118 requirements approved; 10 excluded (gaps AQPI-8, AQPI-13, AQPI-22); 0 conflict(s) resolved</t>
@@ -11241,7 +11241,7 @@
         <v>669</v>
       </c>
       <c r="E2" s="2">
-        <v>1091</v>
+        <v>1197</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -11260,7 +11260,7 @@
         <v>669</v>
       </c>
       <c r="E3" s="2">
-        <v>103</v>
+        <v>118</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -11279,7 +11279,7 @@
         <v>669</v>
       </c>
       <c r="E4" s="2">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -11298,7 +11298,7 @@
         <v>669</v>
       </c>
       <c r="E5" s="2">
-        <v>77</v>
+        <v>98</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -11317,7 +11317,7 @@
         <v>669</v>
       </c>
       <c r="E6" s="2">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -11336,7 +11336,7 @@
         <v>669</v>
       </c>
       <c r="E7" s="2">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -11355,7 +11355,7 @@
         <v>669</v>
       </c>
       <c r="E8" s="2">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -11395,7 +11395,7 @@
         <v>669</v>
       </c>
       <c r="E10" s="2">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>

</xml_diff>